<commit_message>
feat: improve primary site coding
</commit_message>
<xml_diff>
--- a/Laterality.xlsx
+++ b/Laterality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\ePath_to_CRS_Linkage\2024\assign-vars\epath-to-matchpro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904A17FA-695D-4B47-A86D-9E1B1DCBD390}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5535AD-91DF-4CE3-87D8-2BAA45EC8FF1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="450" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="900" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>